<commit_message>
feat(文法形式): 学習倍増(N5 211→398・各点4問)＋模試プール新設(N5:160/N4:150/N3:130=公式×10・全問ユニーク)＋結線(GRAMMAR_FORM_MOCK/HAS_MOCK_POOL)＋番人(grammarFormMock 6件)＋在庫Excel/一意性Excel更新
- 配置: grammar_form_N5 学習+187(N5-G-B-0228〜・各pointId=4問)／新規 content/problems/bunpou/mock/grammar_form_{N5,N4,N3}.json(pool=mock)
- 結線: rehydrate GRAMMAR_FORM_MOCK・index export・daimon(HAS_MOCK_POOL+='grammar_form'/GF_MOCK_INDEX/mockUnitIds/questionForUnit useMock分岐)
- 番人: src/data/grammarFormMock.test.ts(件数/空所1個/4択先頭正解/pointId実在/id帯/stem重複なし)・package.json登録
- 機械修正: 空所マーカーを生成物【　】→アプリ実装前提〔　〕へ全627問変換／既存と完全一致のlearn stem 3件を別文脈へ最小改変(pointId/answer/choices保持)
- 検証: rebuild(84)・tsc0・npm test 458/458・ランタイム実測(mockUnits160/150/130・cloze・空所〔　〕・学習では未解決=汚染なし)
- 在庫Excel: stock_report→mock_stock(bunpou模試換算 N5=24回)→stock_excel(MOCK dict 文法形式160/150/130)→daimon_solvability --xlsx

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memory/在庫・模試ストックまとめ.xlsx
+++ b/memory/在庫・模試ストックまとめ.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② カバー率" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ 品質・攻略耐性" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑥ 翻訳状況" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="聴解攻略耐性分析" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'大問別まとめ'!$A$1:$L$1</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="37">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -239,8 +240,17 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <color rgb="009C6500"/>
+    </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <color rgb="009C0006"/>
+    </font>
   </fonts>
-  <fills count="47">
+  <fills count="49">
     <fill>
       <patternFill/>
     </fill>
@@ -474,6 +484,16 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -604,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -887,6 +907,12 @@
     <xf numFmtId="0" fontId="0" fillId="46" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="46" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="48" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2056,17 +2082,15 @@
         </is>
       </c>
       <c r="D16" s="98" t="n">
-        <v>211</v>
+        <v>398</v>
       </c>
       <c r="E16" s="98" t="inlineStr">
         <is>
           <t>×1</t>
         </is>
       </c>
-      <c r="F16" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F16" s="98" t="n">
+        <v>160</v>
       </c>
       <c r="G16" s="97" t="inlineStr"/>
       <c r="H16" s="98" t="inlineStr">
@@ -2077,12 +2101,12 @@
       <c r="I16" s="98" t="n">
         <v>16</v>
       </c>
-      <c r="J16" s="103" t="n">
-        <v>13</v>
+      <c r="J16" s="100" t="n">
+        <v>24</v>
       </c>
       <c r="K16" s="97" t="inlineStr">
         <is>
-          <t>3:210 / 4:1</t>
+          <t>3:397 / 4:1</t>
         </is>
       </c>
       <c r="L16" s="98" t="inlineStr">
@@ -2115,10 +2139,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F17" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F17" s="98" t="n">
+        <v>150</v>
       </c>
       <c r="G17" s="97" t="inlineStr"/>
       <c r="H17" s="98" t="inlineStr">
@@ -2167,10 +2189,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F18" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="98" t="n">
+        <v>130</v>
       </c>
       <c r="G18" s="97" t="inlineStr"/>
       <c r="H18" s="98" t="inlineStr">
@@ -3730,8 +3750,8 @@
           <t>文法</t>
         </is>
       </c>
-      <c r="B6" s="109" t="n">
-        <v>13</v>
+      <c r="B6" s="108" t="n">
+        <v>24</v>
       </c>
       <c r="C6" s="108" t="n">
         <v>24</v>
@@ -3807,8 +3827,8 @@
           <t>フル模試</t>
         </is>
       </c>
-      <c r="B12" s="103" t="n">
-        <v>13</v>
+      <c r="B12" s="100" t="n">
+        <v>21</v>
       </c>
       <c r="C12" s="100" t="n">
         <v>18</v>
@@ -11254,4 +11274,1212 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="82" min="1" max="1"/>
+    <col width="6" customWidth="1" style="82" min="2" max="2"/>
+    <col width="6" customWidth="1" style="82" min="3" max="3"/>
+    <col width="6" customWidth="1" style="82" min="4" max="4"/>
+    <col width="16" customWidth="1" style="82" min="5" max="5"/>
+    <col width="15" customWidth="1" style="82" min="6" max="6"/>
+    <col width="8" customWidth="1" style="82" min="7" max="7"/>
+    <col width="8" customWidth="1" style="82" min="8" max="8"/>
+    <col width="12" customWidth="1" style="82" min="9" max="9"/>
+    <col width="6" customWidth="1" style="82" min="10" max="10"/>
+    <col width="12" customWidth="1" style="82" min="11" max="11"/>
+    <col width="14" customWidth="1" style="82" min="12" max="12"/>
+    <col width="12" customWidth="1" style="82" min="13" max="13"/>
+    <col width="12" customWidth="1" style="82" min="14" max="14"/>
+    <col width="14" customWidth="1" style="82" min="15" max="15"/>
+    <col width="12" customWidth="1" style="82" min="16" max="16"/>
+    <col width="12" customWidth="1" style="82" min="17" max="17"/>
+    <col width="5" customWidth="1" style="82" min="18" max="18"/>
+    <col width="5" customWidth="1" style="82" min="19" max="19"/>
+    <col width="8" customWidth="1" style="82" min="20" max="20"/>
+    <col width="8" customWidth="1" style="82" min="21" max="21"/>
+    <col width="8" customWidth="1" style="82" min="22" max="22"/>
+    <col width="9" customWidth="1" style="82" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>聴解 攻略耐性・モーラ・ワンパターン 分析（2026-08-16 自動集計｜daimon_solvability.py）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>★セル色＝信号：緑=合格／黄=境界・注意／赤=要改善。しきい値＝最長≤基準+15・語彙マッチ≤基準+10・正誤差≤+1.0・設問テンプレ≤30%・台本/選択肢重複=0・帯外=0が理想・係/留守=0・(発話)依頼形≤35%/形分離≤65%・位置最大≤基準+7。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>本質3観点→ ①答えが本文/設問から予測できる ②誤答が弱い ③大問×レベル内でワンパターン/重複。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>語彙マッチ的中%=「本文と最も語が重なる選択肢」を選ぶと正解になる割合(基準=1/選択肢数)。高い=正解だけ本文語→聞かず語マッチで解ける(①②)。良い設計は正解を言い換え本文語は誤答へ罠として置く。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>正解−誤答 本文一致差=正解の本文一致語数−誤答平均。+大=正解だけ本文語(①②)。最長を選ぶ的中=正解が最長選択肢の割合(②)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>選択肢方式「表示時ランダム」(課題/ポイント/概要=テキスト4択)はアプリが並べ替え→正解位置は無関係(正本①固定でOK)。「音声焼込み」(発話/即時)は位置固定→位置偏りが有効。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>台本重複/選択肢セット重複=同一大問×レベル内の近似(③)。設問テンプレ最大=同一設問文の最大シェア(③)。設計帯:課題/ポイント/概要/発話=公式中央値±20%、即時=公式実測再センタリング。既存問の帯外は帯導入前の据え置き。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="122" t="inlineStr">
+        <is>
+          <t>大問</t>
+        </is>
+      </c>
+      <c r="B8" s="122" t="inlineStr">
+        <is>
+          <t>レベル</t>
+        </is>
+      </c>
+      <c r="C8" s="122" t="inlineStr">
+        <is>
+          <t>問題数</t>
+        </is>
+      </c>
+      <c r="D8" s="122" t="inlineStr">
+        <is>
+          <t>選択肢数</t>
+        </is>
+      </c>
+      <c r="E8" s="122" t="inlineStr">
+        <is>
+          <t>選択肢方式</t>
+        </is>
+      </c>
+      <c r="F8" s="122" t="inlineStr">
+        <is>
+          <t>台本モーラ min/中/max</t>
+        </is>
+      </c>
+      <c r="G8" s="122" t="inlineStr">
+        <is>
+          <t>設計帯</t>
+        </is>
+      </c>
+      <c r="H8" s="122" t="inlineStr">
+        <is>
+          <t>帯外 短/長</t>
+        </is>
+      </c>
+      <c r="I8" s="122" t="inlineStr">
+        <is>
+          <t>最長を選ぶ的中%</t>
+        </is>
+      </c>
+      <c r="J8" s="122" t="inlineStr">
+        <is>
+          <t>基準%</t>
+        </is>
+      </c>
+      <c r="K8" s="122" t="inlineStr">
+        <is>
+          <t>語彙マッチ的中%</t>
+        </is>
+      </c>
+      <c r="L8" s="122" t="inlineStr">
+        <is>
+          <t>正解−誤答 本文一致差</t>
+        </is>
+      </c>
+      <c r="M8" s="122" t="inlineStr">
+        <is>
+          <t>設問テンプレ最大%</t>
+        </is>
+      </c>
+      <c r="N8" s="122" t="inlineStr">
+        <is>
+          <t>台本重複(≥.60)</t>
+        </is>
+      </c>
+      <c r="O8" s="122" t="inlineStr">
+        <is>
+          <t>選択肢セット重複(≥.70)</t>
+        </is>
+      </c>
+      <c r="P8" s="122" t="inlineStr">
+        <is>
+          <t>正解位置(正本)</t>
+        </is>
+      </c>
+      <c r="Q8" s="122" t="inlineStr">
+        <is>
+          <t>位置最大%(有効時)</t>
+        </is>
+      </c>
+      <c r="R8" s="122" t="inlineStr">
+        <is>
+          <t>係</t>
+        </is>
+      </c>
+      <c r="S8" s="122" t="inlineStr">
+        <is>
+          <t>留守</t>
+        </is>
+      </c>
+      <c r="T8" s="122" t="inlineStr">
+        <is>
+          <t>依頼形%</t>
+        </is>
+      </c>
+      <c r="U8" s="122" t="inlineStr">
+        <is>
+          <t>形分離%</t>
+        </is>
+      </c>
+      <c r="V8" s="122" t="inlineStr">
+        <is>
+          <t>機能max%</t>
+        </is>
+      </c>
+      <c r="W8" s="122" t="inlineStr">
+        <is>
+          <t>弁別軸max%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>課題理解</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>150</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>183/306/384</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>258-386</t>
+        </is>
+      </c>
+      <c r="H9" s="123" t="inlineStr">
+        <is>
+          <t>19/0</t>
+        </is>
+      </c>
+      <c r="I9" s="124" t="n">
+        <v>36</v>
+      </c>
+      <c r="J9" t="n">
+        <v>25</v>
+      </c>
+      <c r="K9" s="124" t="n">
+        <v>29</v>
+      </c>
+      <c r="L9" s="124" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M9" s="124" t="n">
+        <v>9</v>
+      </c>
+      <c r="N9" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R9" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>課題理解</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>150</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>163/241/311</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>209-313</t>
+        </is>
+      </c>
+      <c r="H10" s="123" t="inlineStr">
+        <is>
+          <t>20/0</t>
+        </is>
+      </c>
+      <c r="I10" s="124" t="n">
+        <v>34</v>
+      </c>
+      <c r="J10" t="n">
+        <v>25</v>
+      </c>
+      <c r="K10" s="124" t="n">
+        <v>19</v>
+      </c>
+      <c r="L10" s="124" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M10" s="124" t="n">
+        <v>8</v>
+      </c>
+      <c r="N10" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="125" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R10" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>課題理解</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>150</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>73/115/154</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>105-157</t>
+        </is>
+      </c>
+      <c r="H11" s="123" t="inlineStr">
+        <is>
+          <t>18/0</t>
+        </is>
+      </c>
+      <c r="I11" s="124" t="n">
+        <v>38</v>
+      </c>
+      <c r="J11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K11" s="124" t="n">
+        <v>13</v>
+      </c>
+      <c r="L11" s="124" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M11" s="124" t="n">
+        <v>16</v>
+      </c>
+      <c r="N11" s="125" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R11" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ポイント理解</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>150</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>183/239/290</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>179-269</t>
+        </is>
+      </c>
+      <c r="H12" s="123" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="I12" s="123" t="n">
+        <v>45</v>
+      </c>
+      <c r="J12" t="n">
+        <v>25</v>
+      </c>
+      <c r="K12" s="124" t="n">
+        <v>17</v>
+      </c>
+      <c r="L12" s="124" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M12" s="124" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="125" t="n">
+        <v>2</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R12" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ポイント理解</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>150</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>124/196/263</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>175-263</t>
+        </is>
+      </c>
+      <c r="H13" s="123" t="inlineStr">
+        <is>
+          <t>21/0</t>
+        </is>
+      </c>
+      <c r="I13" s="124" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" t="n">
+        <v>25</v>
+      </c>
+      <c r="K13" s="124" t="n">
+        <v>19</v>
+      </c>
+      <c r="L13" s="124" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M13" s="124" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R13" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ポイント理解</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>84/168/216</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>149-223</t>
+        </is>
+      </c>
+      <c r="H14" s="123" t="inlineStr">
+        <is>
+          <t>29/0</t>
+        </is>
+      </c>
+      <c r="I14" s="124" t="n">
+        <v>23</v>
+      </c>
+      <c r="J14" t="n">
+        <v>25</v>
+      </c>
+      <c r="K14" s="124" t="n">
+        <v>10</v>
+      </c>
+      <c r="L14" s="124" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M14" s="124" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>150/0/0/0</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R14" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>概要理解</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>表示時ランダム</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>203/234/272</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>190-284</t>
+        </is>
+      </c>
+      <c r="H15" s="124" t="inlineStr">
+        <is>
+          <t>0/0</t>
+        </is>
+      </c>
+      <c r="I15" s="124" t="n">
+        <v>18</v>
+      </c>
+      <c r="J15" t="n">
+        <v>25</v>
+      </c>
+      <c r="K15" s="124" t="n">
+        <v>10</v>
+      </c>
+      <c r="L15" s="124" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="M15" s="124" t="n">
+        <v>12</v>
+      </c>
+      <c r="N15" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>20/20/20/20</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R15" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>発話表現</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>200</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>29/40/47</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>27-41</t>
+        </is>
+      </c>
+      <c r="H16" s="123" t="inlineStr">
+        <is>
+          <t>0/71</t>
+        </is>
+      </c>
+      <c r="I16" s="124" t="n">
+        <v>28</v>
+      </c>
+      <c r="J16" t="n">
+        <v>33</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>60/74/66</t>
+        </is>
+      </c>
+      <c r="Q16" s="124" t="n">
+        <v>37</v>
+      </c>
+      <c r="R16" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="124" t="n">
+        <v>12</v>
+      </c>
+      <c r="U16" s="124" t="n">
+        <v>56</v>
+      </c>
+      <c r="V16" t="n">
+        <v>33</v>
+      </c>
+      <c r="W16" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>発話表現</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>200</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>24/38/47</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>20-30</t>
+        </is>
+      </c>
+      <c r="H17" s="123" t="inlineStr">
+        <is>
+          <t>0/183</t>
+        </is>
+      </c>
+      <c r="I17" s="124" t="n">
+        <v>28</v>
+      </c>
+      <c r="J17" t="n">
+        <v>33</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>58/74/68</t>
+        </is>
+      </c>
+      <c r="Q17" s="124" t="n">
+        <v>37</v>
+      </c>
+      <c r="R17" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="124" t="n">
+        <v>7</v>
+      </c>
+      <c r="U17" s="124" t="n">
+        <v>54</v>
+      </c>
+      <c r="V17" t="n">
+        <v>28</v>
+      </c>
+      <c r="W17" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>発話表現</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>200</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>24/36/47</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>20-30</t>
+        </is>
+      </c>
+      <c r="H18" s="123" t="inlineStr">
+        <is>
+          <t>0/168</t>
+        </is>
+      </c>
+      <c r="I18" s="124" t="n">
+        <v>32</v>
+      </c>
+      <c r="J18" t="n">
+        <v>33</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>59/77/64</t>
+        </is>
+      </c>
+      <c r="Q18" s="124" t="n">
+        <v>38</v>
+      </c>
+      <c r="R18" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="124" t="n">
+        <v>6</v>
+      </c>
+      <c r="U18" s="124" t="n">
+        <v>50</v>
+      </c>
+      <c r="V18" t="n">
+        <v>26</v>
+      </c>
+      <c r="W18" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>即時応答</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>240</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>13/26/46</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>18-32</t>
+        </is>
+      </c>
+      <c r="H19" s="123" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="I19" s="124" t="n">
+        <v>46</v>
+      </c>
+      <c r="J19" t="n">
+        <v>33</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="125" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>94/74/72</t>
+        </is>
+      </c>
+      <c r="Q19" s="124" t="n">
+        <v>39</v>
+      </c>
+      <c r="R19" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>即時応答</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>240</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>12/25/33</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>18-33</t>
+        </is>
+      </c>
+      <c r="H20" s="123" t="inlineStr">
+        <is>
+          <t>9/0</t>
+        </is>
+      </c>
+      <c r="I20" s="124" t="n">
+        <v>40</v>
+      </c>
+      <c r="J20" t="n">
+        <v>33</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>94/74/72</t>
+        </is>
+      </c>
+      <c r="Q20" s="124" t="n">
+        <v>39</v>
+      </c>
+      <c r="R20" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>即時応答</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>240</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>音声焼込み(位置固定)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>8/24/30</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>14-27</t>
+        </is>
+      </c>
+      <c r="H21" s="123" t="inlineStr">
+        <is>
+          <t>13/21</t>
+        </is>
+      </c>
+      <c r="I21" s="124" t="n">
+        <v>38</v>
+      </c>
+      <c r="J21" t="n">
+        <v>33</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="125" t="n">
+        <v>2</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>94/74/72</t>
+        </is>
+      </c>
+      <c r="Q21" s="124" t="n">
+        <v>39</v>
+      </c>
+      <c r="R21" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(組み立て・文章の文法): 模試プール結線(ORDER_MOCK/PASSAGE_GRAMMAR_MOCK・HAS_MOCK_POOL+order・questionForUnit mock分岐・MockScreen passageGrammar mock優先)＋番人12件(orderMock/passageGrammarMock新設)＋在庫Excel(模試 組み立て/文章の文法 各50×3・割増倍数E19-E24=在庫問題数/辞書文法点数を小数化)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memory/在庫・模試ストックまとめ.xlsx
+++ b/memory/在庫・模試ストックまとめ.xlsx
@@ -2234,15 +2234,13 @@
       <c r="D19" s="98" t="n">
         <v>146</v>
       </c>
-      <c r="E19" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F19" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E19" s="99" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="F19" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G19" s="97" t="inlineStr"/>
       <c r="H19" s="98" t="inlineStr">
@@ -2286,15 +2284,13 @@
       <c r="D20" s="98" t="n">
         <v>216</v>
       </c>
-      <c r="E20" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F20" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E20" s="99" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="F20" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G20" s="97" t="inlineStr"/>
       <c r="H20" s="98" t="inlineStr">
@@ -2338,15 +2334,13 @@
       <c r="D21" s="98" t="n">
         <v>311</v>
       </c>
-      <c r="E21" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F21" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="99" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="F21" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G21" s="97" t="inlineStr"/>
       <c r="H21" s="98" t="inlineStr">
@@ -2390,15 +2384,13 @@
       <c r="D22" s="98" t="n">
         <v>400</v>
       </c>
-      <c r="E22" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F22" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="99" t="inlineStr">
+        <is>
+          <t>4.40</t>
+        </is>
+      </c>
+      <c r="F22" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G22" s="97" t="inlineStr"/>
       <c r="H22" s="98" t="n">
@@ -2440,15 +2432,13 @@
       <c r="D23" s="98" t="n">
         <v>300</v>
       </c>
-      <c r="E23" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F23" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="99" t="inlineStr">
+        <is>
+          <t>2.29</t>
+        </is>
+      </c>
+      <c r="F23" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G23" s="97" t="inlineStr"/>
       <c r="H23" s="98" t="n">
@@ -2490,15 +2480,13 @@
       <c r="D24" s="98" t="n">
         <v>350</v>
       </c>
-      <c r="E24" s="98" t="inlineStr">
-        <is>
-          <t>×1</t>
-        </is>
-      </c>
-      <c r="F24" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E24" s="99" t="inlineStr">
+        <is>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="F24" s="98" t="n">
+        <v>50</v>
       </c>
       <c r="G24" s="97" t="inlineStr"/>
       <c r="H24" s="98" t="n">
@@ -11550,10 +11538,6 @@
       <c r="S9" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11629,10 +11613,6 @@
       <c r="S10" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11708,10 +11688,6 @@
       <c r="S11" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11787,10 +11763,6 @@
       <c r="S12" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11866,10 +11838,6 @@
       <c r="S13" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11945,10 +11913,6 @@
       <c r="S14" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12024,10 +11988,6 @@
       <c r="S15" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12072,9 +12032,6 @@
       <c r="J16" t="n">
         <v>33</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" s="124" t="n">
         <v>0</v>
       </c>
@@ -12151,9 +12108,6 @@
       <c r="J17" t="n">
         <v>33</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" s="124" t="n">
         <v>0</v>
       </c>
@@ -12230,9 +12184,6 @@
       <c r="J18" t="n">
         <v>33</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" s="124" t="n">
         <v>0</v>
       </c>
@@ -12309,9 +12260,6 @@
       <c r="J19" t="n">
         <v>33</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" s="124" t="n">
         <v>0</v>
       </c>
@@ -12332,10 +12280,6 @@
       <c r="S19" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12380,9 +12324,6 @@
       <c r="J20" t="n">
         <v>33</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" s="124" t="n">
         <v>0</v>
       </c>
@@ -12403,10 +12344,6 @@
       <c r="S20" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -12451,9 +12388,6 @@
       <c r="J21" t="n">
         <v>33</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" s="124" t="n">
         <v>0</v>
       </c>
@@ -12474,10 +12408,6 @@
       <c r="S21" s="124" t="n">
         <v>0</v>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(読解): 模試プール新設(内容理解 短/中/長・情報検索 210本文320設問・pool='mock'初見)＋結線(READING_MOCK/readingMockItemsForSub・MockScreen mock優先fallback)＋ルビ(自級以上4156)＋翻訳(joho以外160本文270設問 en/ne・Gemini2.5Flash ¥47)＋番人(readingMock 210/320・passageTransNe を READING_MOCK 含むよう拡張)＋在庫Excel(読解4大問)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/memory/在庫・模試ストックまとめ.xlsx
+++ b/memory/在庫・模試ストックまとめ.xlsx
@@ -2533,10 +2533,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F25" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F25" s="98" t="n">
+        <v>30</v>
       </c>
       <c r="G25" s="97" t="inlineStr"/>
       <c r="H25" s="98" t="n">
@@ -2583,10 +2581,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F26" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F26" s="98" t="n">
+        <v>40</v>
       </c>
       <c r="G26" s="97" t="inlineStr"/>
       <c r="H26" s="98" t="n">
@@ -2633,10 +2629,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F27" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F27" s="98" t="n">
+        <v>40</v>
       </c>
       <c r="G27" s="97" t="inlineStr"/>
       <c r="H27" s="98" t="n">
@@ -2683,10 +2677,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F28" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F28" s="98" t="n">
+        <v>20</v>
       </c>
       <c r="G28" s="97" t="inlineStr"/>
       <c r="H28" s="98" t="n">
@@ -2733,10 +2725,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F29" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F29" s="98" t="n">
+        <v>40</v>
       </c>
       <c r="G29" s="97" t="inlineStr"/>
       <c r="H29" s="98" t="n">
@@ -2783,10 +2773,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F30" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F30" s="98" t="n">
+        <v>60</v>
       </c>
       <c r="G30" s="97" t="inlineStr"/>
       <c r="H30" s="98" t="n">
@@ -2833,10 +2821,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F31" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F31" s="98" t="n">
+        <v>40</v>
       </c>
       <c r="G31" s="97" t="inlineStr"/>
       <c r="H31" s="98" t="n">
@@ -2883,10 +2869,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F32" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F32" s="98" t="n">
+        <v>10</v>
       </c>
       <c r="G32" s="97" t="inlineStr"/>
       <c r="H32" s="98" t="n">
@@ -2933,10 +2917,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F33" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F33" s="98" t="n">
+        <v>20</v>
       </c>
       <c r="G33" s="97" t="inlineStr"/>
       <c r="H33" s="98" t="n">
@@ -2983,10 +2965,8 @@
           <t>×1</t>
         </is>
       </c>
-      <c r="F34" s="98" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F34" s="98" t="n">
+        <v>20</v>
       </c>
       <c r="G34" s="97" t="inlineStr"/>
       <c r="H34" s="98" t="n">

</xml_diff>